<commit_message>
ABD dip hourly update
</commit_message>
<xml_diff>
--- a/dip_yakalama_daily_120dip_rebound_sonuclar.xlsx
+++ b/dip_yakalama_daily_120dip_rebound_sonuclar.xlsx
@@ -661,7 +661,7 @@
         <v>3.25</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.13164</v>
+        <v>-3.13117</v>
       </c>
     </row>
     <row r="11">
@@ -991,13 +991,13 @@
         <v>438.53</v>
       </c>
       <c r="D24" t="n">
-        <v>466.62</v>
+        <v>465.88</v>
       </c>
       <c r="E24" t="n">
-        <v>6.41</v>
+        <v>6.24</v>
       </c>
       <c r="F24" t="n">
-        <v>2.31573</v>
+        <v>1.59844</v>
       </c>
     </row>
     <row r="25">
@@ -1405,7 +1405,7 @@
         <v>6.48</v>
       </c>
       <c r="F41" t="n">
-        <v>1.5016</v>
+        <v>2.71573</v>
       </c>
     </row>
     <row r="42">
@@ -2479,13 +2479,13 @@
         <v>76.53</v>
       </c>
       <c r="D86" t="n">
-        <v>95.78</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="E86" t="n">
-        <v>25.15</v>
+        <v>24.92</v>
       </c>
       <c r="F86" t="n">
-        <v>0.37222</v>
+        <v>0.14719</v>
       </c>
     </row>
     <row r="87">
@@ -4117,7 +4117,7 @@
         <v>42.87</v>
       </c>
       <c r="F154" t="n">
-        <v>1.46722</v>
+        <v>1.32749</v>
       </c>
     </row>
     <row r="155">
@@ -4147,7 +4147,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>LTM</t>
+          <t>MMM</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4156,22 +4156,22 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>45.26</v>
+        <v>141.56</v>
       </c>
       <c r="D156" t="n">
-        <v>52.45</v>
+        <v>169.55</v>
       </c>
       <c r="E156" t="n">
-        <v>15.89</v>
+        <v>19.77</v>
       </c>
       <c r="F156" t="n">
-        <v>0.28353</v>
+        <v>0.30115</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SCCO</t>
+          <t>LTM</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4180,22 +4180,22 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>162.7</v>
+        <v>45.26</v>
       </c>
       <c r="D157" t="n">
-        <v>203.92</v>
+        <v>52.45</v>
       </c>
       <c r="E157" t="n">
-        <v>25.33</v>
+        <v>15.89</v>
       </c>
       <c r="F157" t="n">
-        <v>1.87985</v>
+        <v>0.28353</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>WTS</t>
+          <t>SCCO</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4204,22 +4204,22 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>289.93</v>
+        <v>162.7</v>
       </c>
       <c r="D158" t="n">
-        <v>357.79</v>
+        <v>203.92</v>
       </c>
       <c r="E158" t="n">
-        <v>23.41</v>
+        <v>25.33</v>
       </c>
       <c r="F158" t="n">
-        <v>-0.35666</v>
+        <v>1.87985</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>WTS</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4228,22 +4228,22 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>55.57</v>
+        <v>289.93</v>
       </c>
       <c r="D159" t="n">
-        <v>72.31</v>
+        <v>357.79</v>
       </c>
       <c r="E159" t="n">
-        <v>30.12</v>
+        <v>23.41</v>
       </c>
       <c r="F159" t="n">
-        <v>0.30707</v>
+        <v>-0.35666</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4252,22 +4252,22 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>323.85</v>
+        <v>55.57</v>
       </c>
       <c r="D160" t="n">
-        <v>414.61</v>
+        <v>72.31</v>
       </c>
       <c r="E160" t="n">
-        <v>28.03</v>
+        <v>30.12</v>
       </c>
       <c r="F160" t="n">
-        <v>3.0944</v>
+        <v>0.30707</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>BBVA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4276,22 +4276,22 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>141.56</v>
+        <v>20.83</v>
       </c>
       <c r="D161" t="n">
-        <v>169.55</v>
+        <v>28.87</v>
       </c>
       <c r="E161" t="n">
-        <v>19.77</v>
+        <v>38.6</v>
       </c>
       <c r="F161" t="n">
-        <v>0.30115</v>
+        <v>-0.08143</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BBVA</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4300,22 +4300,22 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>20.83</v>
+        <v>323.85</v>
       </c>
       <c r="D162" t="n">
-        <v>28.87</v>
+        <v>414.61</v>
       </c>
       <c r="E162" t="n">
-        <v>38.6</v>
+        <v>28.03</v>
       </c>
       <c r="F162" t="n">
-        <v>-0.08143</v>
+        <v>3.0944</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>AES</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4324,22 +4324,22 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>14.28</v>
+        <v>45.37</v>
       </c>
       <c r="D163" t="n">
-        <v>14.87</v>
+        <v>198.88</v>
       </c>
       <c r="E163" t="n">
-        <v>4.13</v>
+        <v>338.35</v>
       </c>
       <c r="F163" t="n">
-        <v>0.01483</v>
+        <v>16.38788</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>AES</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4348,16 +4348,16 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>45.37</v>
+        <v>14.28</v>
       </c>
       <c r="D164" t="n">
-        <v>198.88</v>
+        <v>14.87</v>
       </c>
       <c r="E164" t="n">
-        <v>338.35</v>
+        <v>4.13</v>
       </c>
       <c r="F164" t="n">
-        <v>16.38788</v>
+        <v>0.01483</v>
       </c>
     </row>
     <row r="165">
@@ -4483,7 +4483,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4492,22 +4492,22 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>851.21</v>
+        <v>423.24</v>
       </c>
       <c r="D170" t="n">
-        <v>1183.46</v>
+        <v>526.1900000000001</v>
       </c>
       <c r="E170" t="n">
-        <v>39.03</v>
+        <v>24.32</v>
       </c>
       <c r="F170" t="n">
-        <v>4.9927</v>
+        <v>-0.76747</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>WAT</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4516,22 +4516,22 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>292.13</v>
+        <v>851.21</v>
       </c>
       <c r="D171" t="n">
-        <v>433.54</v>
+        <v>1183.46</v>
       </c>
       <c r="E171" t="n">
-        <v>48.41</v>
+        <v>39.03</v>
       </c>
       <c r="F171" t="n">
-        <v>4.8482</v>
+        <v>4.9927</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>WAT</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4540,16 +4540,16 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>423.24</v>
+        <v>292.13</v>
       </c>
       <c r="D172" t="n">
-        <v>526.1900000000001</v>
+        <v>433.54</v>
       </c>
       <c r="E172" t="n">
-        <v>24.32</v>
+        <v>48.41</v>
       </c>
       <c r="F172" t="n">
-        <v>-0.76747</v>
+        <v>4.8482</v>
       </c>
     </row>
     <row r="173">
@@ -4915,7 +4915,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>VLO</t>
+          <t>MPC</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -4924,22 +4924,22 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>223.65</v>
+        <v>213.69</v>
       </c>
       <c r="D188" t="n">
-        <v>387.18</v>
+        <v>393.52</v>
       </c>
       <c r="E188" t="n">
-        <v>73.12</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="F188" t="n">
-        <v>0.84278</v>
+        <v>0.05798</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>MPC</t>
+          <t>VLO</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -4948,16 +4948,16 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>213.69</v>
+        <v>223.65</v>
       </c>
       <c r="D189" t="n">
-        <v>393.52</v>
+        <v>387.18</v>
       </c>
       <c r="E189" t="n">
-        <v>84.15000000000001</v>
+        <v>73.12</v>
       </c>
       <c r="F189" t="n">
-        <v>0.05798</v>
+        <v>0.84278</v>
       </c>
     </row>
     <row r="190">
@@ -5035,7 +5035,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5044,16 +5044,16 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>32.36</v>
+        <v>121.11</v>
       </c>
       <c r="D193" t="n">
-        <v>57.95</v>
+        <v>335.94</v>
       </c>
       <c r="E193" t="n">
-        <v>79.08</v>
+        <v>177.38</v>
       </c>
       <c r="F193" t="n">
-        <v>1.75702</v>
+        <v>2.00858</v>
       </c>
     </row>
     <row r="194">
@@ -5083,7 +5083,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5092,22 +5092,22 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>118.05</v>
+        <v>32.36</v>
       </c>
       <c r="D195" t="n">
-        <v>193.05</v>
+        <v>57.95</v>
       </c>
       <c r="E195" t="n">
-        <v>63.53</v>
+        <v>79.08</v>
       </c>
       <c r="F195" t="n">
-        <v>8.029579999999999</v>
+        <v>1.75702</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>HUM</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5116,22 +5116,22 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>225.95</v>
+        <v>192.15</v>
       </c>
       <c r="D196" t="n">
-        <v>410.44</v>
+        <v>397.93</v>
       </c>
       <c r="E196" t="n">
-        <v>81.65000000000001</v>
+        <v>107.09</v>
       </c>
       <c r="F196" t="n">
-        <v>10.18926</v>
+        <v>-3.04898</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5140,22 +5140,22 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>289.81</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="D197" t="n">
-        <v>443.06</v>
+        <v>177.25</v>
       </c>
       <c r="E197" t="n">
-        <v>52.88</v>
+        <v>125.51</v>
       </c>
       <c r="F197" t="n">
-        <v>11.78253</v>
+        <v>2.85042</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5164,22 +5164,22 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>121.11</v>
+        <v>289.81</v>
       </c>
       <c r="D198" t="n">
-        <v>335.94</v>
+        <v>443.06</v>
       </c>
       <c r="E198" t="n">
-        <v>177.38</v>
+        <v>52.88</v>
       </c>
       <c r="F198" t="n">
-        <v>2.00858</v>
+        <v>11.78253</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5188,22 +5188,22 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>57.15</v>
+        <v>265.66</v>
       </c>
       <c r="D199" t="n">
-        <v>187.74</v>
+        <v>326.13</v>
       </c>
       <c r="E199" t="n">
-        <v>228.5</v>
+        <v>22.76</v>
       </c>
       <c r="F199" t="n">
-        <v>3.10412</v>
+        <v>5.91492</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HUM</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5212,22 +5212,22 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>192.15</v>
+        <v>57.15</v>
       </c>
       <c r="D200" t="n">
-        <v>397.93</v>
+        <v>187.74</v>
       </c>
       <c r="E200" t="n">
-        <v>107.09</v>
+        <v>228.5</v>
       </c>
       <c r="F200" t="n">
-        <v>-3.04898</v>
+        <v>3.10412</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>VEEV</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5236,22 +5236,22 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>151.43</v>
+        <v>62.93</v>
       </c>
       <c r="D201" t="n">
-        <v>280.68</v>
+        <v>195.19</v>
       </c>
       <c r="E201" t="n">
-        <v>85.34999999999999</v>
+        <v>210.17</v>
       </c>
       <c r="F201" t="n">
-        <v>3.85236</v>
+        <v>9.40362</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5260,22 +5260,22 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>265.66</v>
+        <v>225.95</v>
       </c>
       <c r="D202" t="n">
-        <v>326.13</v>
+        <v>410.44</v>
       </c>
       <c r="E202" t="n">
-        <v>22.76</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="F202" t="n">
-        <v>5.91492</v>
+        <v>10.18926</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5284,22 +5284,22 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>62.93</v>
+        <v>118.05</v>
       </c>
       <c r="D203" t="n">
-        <v>195.19</v>
+        <v>193.05</v>
       </c>
       <c r="E203" t="n">
-        <v>210.17</v>
+        <v>63.53</v>
       </c>
       <c r="F203" t="n">
-        <v>9.40362</v>
+        <v>8.029579999999999</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>VEEV</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5308,16 +5308,16 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>78.59999999999999</v>
+        <v>151.43</v>
       </c>
       <c r="D204" t="n">
-        <v>177.25</v>
+        <v>280.68</v>
       </c>
       <c r="E204" t="n">
-        <v>125.51</v>
+        <v>85.34999999999999</v>
       </c>
       <c r="F204" t="n">
-        <v>2.85042</v>
+        <v>3.85236</v>
       </c>
     </row>
     <row r="205">
@@ -5347,7 +5347,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5356,22 +5356,22 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>166.99</v>
+        <v>155.73</v>
       </c>
       <c r="D206" t="n">
-        <v>349.02</v>
+        <v>374.74</v>
       </c>
       <c r="E206" t="n">
-        <v>109.01</v>
+        <v>140.63</v>
       </c>
       <c r="F206" t="n">
-        <v>13.69488</v>
+        <v>8.0283</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5380,22 +5380,22 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>155.73</v>
+        <v>166.99</v>
       </c>
       <c r="D207" t="n">
-        <v>374.74</v>
+        <v>349.02</v>
       </c>
       <c r="E207" t="n">
-        <v>140.63</v>
+        <v>109.01</v>
       </c>
       <c r="F207" t="n">
-        <v>8.0283</v>
+        <v>13.69488</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5404,16 +5404,16 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>34.41</v>
+        <v>94.75</v>
       </c>
       <c r="D208" t="n">
-        <v>68.03</v>
+        <v>252.13</v>
       </c>
       <c r="E208" t="n">
-        <v>97.7</v>
+        <v>166.09</v>
       </c>
       <c r="F208" t="n">
-        <v>0.44166</v>
+        <v>10.67113</v>
       </c>
     </row>
     <row r="209">
@@ -5443,7 +5443,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5452,16 +5452,16 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>94.75</v>
+        <v>34.41</v>
       </c>
       <c r="D210" t="n">
-        <v>252.13</v>
+        <v>68.03</v>
       </c>
       <c r="E210" t="n">
-        <v>166.09</v>
+        <v>97.7</v>
       </c>
       <c r="F210" t="n">
-        <v>10.67113</v>
+        <v>0.44166</v>
       </c>
     </row>
     <row r="211">
@@ -5515,7 +5515,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>RBRK</t>
+          <t>TWLO</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5524,22 +5524,22 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>43.81</v>
+        <v>117.65</v>
       </c>
       <c r="D213" t="n">
-        <v>109.55</v>
+        <v>275.8</v>
       </c>
       <c r="E213" t="n">
-        <v>150.06</v>
+        <v>134.42</v>
       </c>
       <c r="F213" t="n">
-        <v>4.67712</v>
+        <v>16.79812</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>TWLO</t>
+          <t>EQH</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5548,22 +5548,22 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>117.65</v>
+        <v>37.43</v>
       </c>
       <c r="D214" t="n">
-        <v>275.8</v>
+        <v>53.84</v>
       </c>
       <c r="E214" t="n">
-        <v>134.42</v>
+        <v>43.84</v>
       </c>
       <c r="F214" t="n">
-        <v>16.79812</v>
+        <v>0.11369</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>EQH</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5572,22 +5572,22 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>37.43</v>
+        <v>69.19</v>
       </c>
       <c r="D215" t="n">
-        <v>53.84</v>
+        <v>119.4</v>
       </c>
       <c r="E215" t="n">
-        <v>43.84</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="F215" t="n">
-        <v>0.11369</v>
+        <v>3.39581</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5596,22 +5596,22 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>69.19</v>
+        <v>76.7</v>
       </c>
       <c r="D216" t="n">
-        <v>119.4</v>
+        <v>173.46</v>
       </c>
       <c r="E216" t="n">
-        <v>72.56999999999999</v>
+        <v>126.15</v>
       </c>
       <c r="F216" t="n">
-        <v>3.39581</v>
+        <v>3.80666</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>RBRK</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5620,16 +5620,16 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>76.7</v>
+        <v>43.81</v>
       </c>
       <c r="D217" t="n">
-        <v>173.46</v>
+        <v>109.55</v>
       </c>
       <c r="E217" t="n">
-        <v>126.15</v>
+        <v>150.06</v>
       </c>
       <c r="F217" t="n">
-        <v>3.80666</v>
+        <v>4.67712</v>
       </c>
     </row>
     <row r="218">
@@ -5659,7 +5659,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5668,22 +5668,22 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>95.67</v>
+        <v>96.22</v>
       </c>
       <c r="D219" t="n">
-        <v>201.15</v>
+        <v>204.97</v>
       </c>
       <c r="E219" t="n">
-        <v>110.25</v>
+        <v>113.02</v>
       </c>
       <c r="F219" t="n">
-        <v>2.03169</v>
+        <v>-1.54484</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5692,22 +5692,22 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>56.43</v>
+        <v>95.67</v>
       </c>
       <c r="D220" t="n">
-        <v>106.82</v>
+        <v>201.15</v>
       </c>
       <c r="E220" t="n">
-        <v>89.3</v>
+        <v>110.25</v>
       </c>
       <c r="F220" t="n">
-        <v>0.04705</v>
+        <v>2.03217</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>DINO</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5716,22 +5716,22 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>96.22</v>
+        <v>56.43</v>
       </c>
       <c r="D221" t="n">
-        <v>204.97</v>
+        <v>106.82</v>
       </c>
       <c r="E221" t="n">
-        <v>113.02</v>
+        <v>89.3</v>
       </c>
       <c r="F221" t="n">
-        <v>-1.54484</v>
+        <v>0.04705</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5740,22 +5740,22 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>96.84</v>
+        <v>199.74</v>
       </c>
       <c r="D222" t="n">
-        <v>128.05</v>
+        <v>278.07</v>
       </c>
       <c r="E222" t="n">
-        <v>32.23</v>
+        <v>39.22</v>
       </c>
       <c r="F222" t="n">
-        <v>3.04814</v>
+        <v>3.0385</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5764,22 +5764,22 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>199.74</v>
+        <v>133.64</v>
       </c>
       <c r="D223" t="n">
-        <v>278.07</v>
+        <v>206.55</v>
       </c>
       <c r="E223" t="n">
-        <v>39.22</v>
+        <v>54.56</v>
       </c>
       <c r="F223" t="n">
-        <v>3.0385</v>
+        <v>3.43321</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5788,16 +5788,16 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>133.64</v>
+        <v>96.84</v>
       </c>
       <c r="D224" t="n">
-        <v>206.55</v>
+        <v>128.05</v>
       </c>
       <c r="E224" t="n">
-        <v>54.56</v>
+        <v>32.23</v>
       </c>
       <c r="F224" t="n">
-        <v>3.43321</v>
+        <v>3.04814</v>
       </c>
     </row>
     <row r="225">
@@ -5851,7 +5851,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -5860,16 +5860,16 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>377.58</v>
+        <v>154.88</v>
       </c>
       <c r="D227" t="n">
-        <v>1082.28</v>
+        <v>187.92</v>
       </c>
       <c r="E227" t="n">
-        <v>186.64</v>
+        <v>21.33</v>
       </c>
       <c r="F227" t="n">
-        <v>37.71915</v>
+        <v>2.79526</v>
       </c>
     </row>
     <row r="228">
@@ -6091,7 +6091,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>AAL</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -6100,22 +6100,22 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>10.81</v>
+        <v>377.58</v>
       </c>
       <c r="D237" t="n">
-        <v>13.87</v>
+        <v>1082.28</v>
       </c>
       <c r="E237" t="n">
-        <v>28.31</v>
+        <v>186.64</v>
       </c>
       <c r="F237" t="n">
-        <v>0.07335999999999999</v>
+        <v>37.71915</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>AAL</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -6124,16 +6124,16 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>154.88</v>
+        <v>10.81</v>
       </c>
       <c r="D238" t="n">
-        <v>187.92</v>
+        <v>13.87</v>
       </c>
       <c r="E238" t="n">
-        <v>21.33</v>
+        <v>28.31</v>
       </c>
       <c r="F238" t="n">
-        <v>2.79526</v>
+        <v>0.07335999999999999</v>
       </c>
     </row>
     <row r="239">
@@ -6187,7 +6187,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>MOG-B</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -6196,22 +6196,22 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>724.4400000000001</v>
+        <v>298.49</v>
       </c>
       <c r="D241" t="n">
-        <v>821.58</v>
+        <v>392.72</v>
       </c>
       <c r="E241" t="n">
-        <v>13.41</v>
+        <v>31.57</v>
       </c>
       <c r="F241" t="n">
-        <v>0.89747</v>
+        <v>3.61037</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6220,22 +6220,22 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>117.13</v>
+        <v>724.4400000000001</v>
       </c>
       <c r="D242" t="n">
-        <v>134.28</v>
+        <v>821.58</v>
       </c>
       <c r="E242" t="n">
-        <v>14.64</v>
+        <v>13.41</v>
       </c>
       <c r="F242" t="n">
-        <v>-0.70935</v>
+        <v>0.89747</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -6244,22 +6244,22 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>224.35</v>
+        <v>117.13</v>
       </c>
       <c r="D243" t="n">
-        <v>315.21</v>
+        <v>134.28</v>
       </c>
       <c r="E243" t="n">
-        <v>40.5</v>
+        <v>14.64</v>
       </c>
       <c r="F243" t="n">
-        <v>4.93703</v>
+        <v>-0.70935</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6268,22 +6268,22 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>131.82</v>
+        <v>224.35</v>
       </c>
       <c r="D244" t="n">
-        <v>224.77</v>
+        <v>315.21</v>
       </c>
       <c r="E244" t="n">
-        <v>70.51000000000001</v>
+        <v>40.5</v>
       </c>
       <c r="F244" t="n">
-        <v>7.14963</v>
+        <v>4.93703</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>SANM</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6292,22 +6292,22 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>354.31</v>
+        <v>131.82</v>
       </c>
       <c r="D245" t="n">
-        <v>485</v>
+        <v>224.77</v>
       </c>
       <c r="E245" t="n">
-        <v>36.89</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="F245" t="n">
-        <v>6.88019</v>
+        <v>7.14963</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6316,22 +6316,22 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>52.91</v>
+        <v>354.31</v>
       </c>
       <c r="D246" t="n">
-        <v>123</v>
+        <v>485</v>
       </c>
       <c r="E246" t="n">
-        <v>132.47</v>
+        <v>36.89</v>
       </c>
       <c r="F246" t="n">
-        <v>7.54484</v>
+        <v>6.88019</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>AIT</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6340,22 +6340,22 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>272.54</v>
+        <v>52.91</v>
       </c>
       <c r="D247" t="n">
-        <v>333.39</v>
+        <v>123</v>
       </c>
       <c r="E247" t="n">
-        <v>22.33</v>
+        <v>132.47</v>
       </c>
       <c r="F247" t="n">
-        <v>2.26361</v>
+        <v>7.54484</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>AIT</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6364,22 +6364,22 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>124.07</v>
+        <v>272.54</v>
       </c>
       <c r="D248" t="n">
-        <v>201.97</v>
+        <v>333.39</v>
       </c>
       <c r="E248" t="n">
-        <v>62.79</v>
+        <v>22.33</v>
       </c>
       <c r="F248" t="n">
-        <v>6.95491</v>
+        <v>2.26361</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6388,22 +6388,22 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>311.96</v>
+        <v>124.07</v>
       </c>
       <c r="D249" t="n">
-        <v>456.81</v>
+        <v>201.97</v>
       </c>
       <c r="E249" t="n">
-        <v>46.43</v>
+        <v>62.79</v>
       </c>
       <c r="F249" t="n">
-        <v>3.49424</v>
+        <v>6.95491</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6412,22 +6412,22 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>327.41</v>
+        <v>311.96</v>
       </c>
       <c r="D250" t="n">
-        <v>393.6</v>
+        <v>456.81</v>
       </c>
       <c r="E250" t="n">
-        <v>20.22</v>
+        <v>46.43</v>
       </c>
       <c r="F250" t="n">
-        <v>6.40618</v>
+        <v>3.49424</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6436,22 +6436,22 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>63.79</v>
+        <v>327.41</v>
       </c>
       <c r="D251" t="n">
-        <v>77.2</v>
+        <v>393.6</v>
       </c>
       <c r="E251" t="n">
-        <v>21.02</v>
+        <v>20.22</v>
       </c>
       <c r="F251" t="n">
-        <v>0.5979</v>
+        <v>6.40618</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>IHG</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6460,22 +6460,22 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>132.02</v>
+        <v>63.79</v>
       </c>
       <c r="D252" t="n">
-        <v>158.16</v>
+        <v>77.2</v>
       </c>
       <c r="E252" t="n">
-        <v>19.8</v>
+        <v>21.02</v>
       </c>
       <c r="F252" t="n">
-        <v>0.18213</v>
+        <v>0.5979</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>IHG</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6484,22 +6484,22 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>71.2</v>
+        <v>132.02</v>
       </c>
       <c r="D253" t="n">
-        <v>97.7</v>
+        <v>158.16</v>
       </c>
       <c r="E253" t="n">
-        <v>37.22</v>
+        <v>19.8</v>
       </c>
       <c r="F253" t="n">
-        <v>0.1183</v>
+        <v>0.18213</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>AME</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6508,22 +6508,22 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>217.75</v>
+        <v>71.2</v>
       </c>
       <c r="D254" t="n">
-        <v>250.74</v>
+        <v>97.7</v>
       </c>
       <c r="E254" t="n">
-        <v>15.15</v>
+        <v>37.22</v>
       </c>
       <c r="F254" t="n">
-        <v>3.22339</v>
+        <v>0.1183</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>ROK</t>
+          <t>AME</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6532,22 +6532,22 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>369.37</v>
+        <v>217.75</v>
       </c>
       <c r="D255" t="n">
-        <v>434.15</v>
+        <v>250.74</v>
       </c>
       <c r="E255" t="n">
-        <v>17.54</v>
+        <v>15.15</v>
       </c>
       <c r="F255" t="n">
-        <v>2.19049</v>
+        <v>3.22339</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>ROK</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6556,22 +6556,22 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>117.4</v>
+        <v>369.37</v>
       </c>
       <c r="D256" t="n">
-        <v>237.33</v>
+        <v>434.15</v>
       </c>
       <c r="E256" t="n">
-        <v>102.16</v>
+        <v>17.54</v>
       </c>
       <c r="F256" t="n">
-        <v>5.22177</v>
+        <v>2.19049</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6580,22 +6580,22 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>106.79</v>
+        <v>117.4</v>
       </c>
       <c r="D257" t="n">
-        <v>210.97</v>
+        <v>237.33</v>
       </c>
       <c r="E257" t="n">
-        <v>97.56</v>
+        <v>102.16</v>
       </c>
       <c r="F257" t="n">
-        <v>4.74621</v>
+        <v>5.22177</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6604,22 +6604,22 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>65.62</v>
+        <v>106.79</v>
       </c>
       <c r="D258" t="n">
-        <v>84.94</v>
+        <v>210.97</v>
       </c>
       <c r="E258" t="n">
-        <v>29.44</v>
+        <v>97.56</v>
       </c>
       <c r="F258" t="n">
-        <v>0.90935</v>
+        <v>4.74621</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6628,22 +6628,22 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>68.20999999999999</v>
+        <v>65.62</v>
       </c>
       <c r="D259" t="n">
-        <v>114.68</v>
+        <v>84.94</v>
       </c>
       <c r="E259" t="n">
-        <v>68.13</v>
+        <v>29.44</v>
       </c>
       <c r="F259" t="n">
-        <v>0.73175</v>
+        <v>0.90935</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6652,22 +6652,22 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>22.19</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="D260" t="n">
-        <v>44.31</v>
+        <v>114.68</v>
       </c>
       <c r="E260" t="n">
-        <v>99.68000000000001</v>
+        <v>68.13</v>
       </c>
       <c r="F260" t="n">
-        <v>1.68906</v>
+        <v>0.73175</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6676,22 +6676,22 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>67.51000000000001</v>
+        <v>22.19</v>
       </c>
       <c r="D261" t="n">
-        <v>78.69</v>
+        <v>44.31</v>
       </c>
       <c r="E261" t="n">
-        <v>16.56</v>
+        <v>99.68000000000001</v>
       </c>
       <c r="F261" t="n">
-        <v>0.91758</v>
+        <v>1.68906</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ZBRA</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6700,22 +6700,22 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>212.51</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="D262" t="n">
-        <v>370.04</v>
+        <v>78.69</v>
       </c>
       <c r="E262" t="n">
-        <v>74.13</v>
+        <v>16.56</v>
       </c>
       <c r="F262" t="n">
-        <v>5.946</v>
+        <v>0.91758</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>STM</t>
+          <t>ZBRA</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6724,22 +6724,22 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>35.68</v>
+        <v>212.51</v>
       </c>
       <c r="D263" t="n">
-        <v>51.93</v>
+        <v>370.04</v>
       </c>
       <c r="E263" t="n">
-        <v>45.54</v>
+        <v>74.13</v>
       </c>
       <c r="F263" t="n">
-        <v>0.54437</v>
+        <v>5.946</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>STM</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6748,22 +6748,22 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1424.91</v>
+        <v>35.68</v>
       </c>
       <c r="D264" t="n">
-        <v>1658.91</v>
+        <v>51.93</v>
       </c>
       <c r="E264" t="n">
-        <v>16.42</v>
+        <v>45.54</v>
       </c>
       <c r="F264" t="n">
-        <v>6.37271</v>
+        <v>0.54437</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>JBL</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6772,22 +6772,22 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>272.85</v>
+        <v>1424.91</v>
       </c>
       <c r="D265" t="n">
-        <v>316.74</v>
+        <v>1658.91</v>
       </c>
       <c r="E265" t="n">
-        <v>16.09</v>
+        <v>16.42</v>
       </c>
       <c r="F265" t="n">
-        <v>1.30767</v>
+        <v>6.37271</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>HMC</t>
+          <t>JBL</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6796,22 +6796,22 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>23.49</v>
+        <v>272.85</v>
       </c>
       <c r="D266" t="n">
-        <v>32.93</v>
+        <v>316.74</v>
       </c>
       <c r="E266" t="n">
-        <v>40.19</v>
+        <v>16.09</v>
       </c>
       <c r="F266" t="n">
-        <v>0.13533</v>
+        <v>1.30767</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>HMC</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -6820,22 +6820,22 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>25.47</v>
+        <v>23.49</v>
       </c>
       <c r="D267" t="n">
-        <v>31.95</v>
+        <v>32.93</v>
       </c>
       <c r="E267" t="n">
-        <v>25.44</v>
+        <v>40.19</v>
       </c>
       <c r="F267" t="n">
-        <v>-0.00395</v>
+        <v>0.13533</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>KDP</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -6844,22 +6844,22 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>118.99</v>
+        <v>25.47</v>
       </c>
       <c r="D268" t="n">
-        <v>364.62</v>
+        <v>31.95</v>
       </c>
       <c r="E268" t="n">
-        <v>206.43</v>
+        <v>25.44</v>
       </c>
       <c r="F268" t="n">
-        <v>22.63037</v>
+        <v>-0.00395</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>TEVA</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -6868,22 +6868,22 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>29.33</v>
+        <v>118.99</v>
       </c>
       <c r="D269" t="n">
-        <v>39.19</v>
+        <v>364.62</v>
       </c>
       <c r="E269" t="n">
-        <v>33.62</v>
+        <v>206.43</v>
       </c>
       <c r="F269" t="n">
-        <v>0.58114</v>
+        <v>22.63037</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>TEVA</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -6892,22 +6892,22 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>9.31</v>
+        <v>29.33</v>
       </c>
       <c r="D270" t="n">
-        <v>24.31</v>
+        <v>39.19</v>
       </c>
       <c r="E270" t="n">
-        <v>161.12</v>
+        <v>33.62</v>
       </c>
       <c r="F270" t="n">
-        <v>0.892</v>
+        <v>0.58114</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -6916,22 +6916,22 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>303.93</v>
+        <v>9.31</v>
       </c>
       <c r="D271" t="n">
-        <v>341.08</v>
+        <v>24.31</v>
       </c>
       <c r="E271" t="n">
-        <v>12.22</v>
+        <v>161.12</v>
       </c>
       <c r="F271" t="n">
-        <v>-0.15355</v>
+        <v>0.892</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -6940,22 +6940,22 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>22.67</v>
+        <v>303.93</v>
       </c>
       <c r="D272" t="n">
-        <v>43.26</v>
+        <v>341.08</v>
       </c>
       <c r="E272" t="n">
-        <v>90.81999999999999</v>
+        <v>12.22</v>
       </c>
       <c r="F272" t="n">
-        <v>1.36575</v>
+        <v>-0.15355</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -6964,22 +6964,22 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>195.12</v>
+        <v>22.67</v>
       </c>
       <c r="D273" t="n">
-        <v>238.08</v>
+        <v>43.26</v>
       </c>
       <c r="E273" t="n">
-        <v>22.02</v>
+        <v>90.81999999999999</v>
       </c>
       <c r="F273" t="n">
-        <v>2.33082</v>
+        <v>1.36575</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>URI</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -6988,22 +6988,22 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>732.74</v>
+        <v>195.12</v>
       </c>
       <c r="D274" t="n">
-        <v>1047.06</v>
+        <v>238.08</v>
       </c>
       <c r="E274" t="n">
-        <v>42.9</v>
+        <v>22.02</v>
       </c>
       <c r="F274" t="n">
-        <v>3.6806</v>
+        <v>2.33082</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>URI</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7012,22 +7012,22 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>265.47</v>
+        <v>732.74</v>
       </c>
       <c r="D275" t="n">
-        <v>325.77</v>
+        <v>1047.06</v>
       </c>
       <c r="E275" t="n">
-        <v>22.71</v>
+        <v>42.9</v>
       </c>
       <c r="F275" t="n">
-        <v>2.91075</v>
+        <v>3.6806</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>HST</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -7036,22 +7036,22 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>19.09</v>
+        <v>118.92</v>
       </c>
       <c r="D276" t="n">
-        <v>22.42</v>
+        <v>164.41</v>
       </c>
       <c r="E276" t="n">
-        <v>17.44</v>
+        <v>38.25</v>
       </c>
       <c r="F276" t="n">
-        <v>-0.0052</v>
+        <v>2.81053</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>HST</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -7060,22 +7060,22 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>143.86</v>
+        <v>19.09</v>
       </c>
       <c r="D277" t="n">
-        <v>310.32</v>
+        <v>22.42</v>
       </c>
       <c r="E277" t="n">
-        <v>115.71</v>
+        <v>17.44</v>
       </c>
       <c r="F277" t="n">
-        <v>19.16082</v>
+        <v>-0.0052</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>SOLV</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -7084,22 +7084,22 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>62.49</v>
+        <v>143.86</v>
       </c>
       <c r="D278" t="n">
-        <v>89.5</v>
+        <v>310.32</v>
       </c>
       <c r="E278" t="n">
-        <v>43.22</v>
+        <v>115.71</v>
       </c>
       <c r="F278" t="n">
-        <v>-0.06796000000000001</v>
+        <v>19.16082</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>WCC</t>
+          <t>SOLV</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7108,22 +7108,22 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>278.57</v>
+        <v>62.49</v>
       </c>
       <c r="D279" t="n">
-        <v>367.44</v>
+        <v>89.5</v>
       </c>
       <c r="E279" t="n">
-        <v>31.9</v>
+        <v>43.22</v>
       </c>
       <c r="F279" t="n">
-        <v>6.33168</v>
+        <v>-0.06796000000000001</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>BNS</t>
+          <t>WCC</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7132,22 +7132,22 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>69.90000000000001</v>
+        <v>278.57</v>
       </c>
       <c r="D280" t="n">
-        <v>93.48</v>
+        <v>367.44</v>
       </c>
       <c r="E280" t="n">
-        <v>33.73</v>
+        <v>31.9</v>
       </c>
       <c r="F280" t="n">
-        <v>0.08166</v>
+        <v>6.33168</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>BNS</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7156,22 +7156,22 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>242.05</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D281" t="n">
-        <v>271.7</v>
+        <v>93.48</v>
       </c>
       <c r="E281" t="n">
-        <v>12.25</v>
+        <v>33.73</v>
       </c>
       <c r="F281" t="n">
-        <v>0.65637</v>
+        <v>0.08166</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7180,22 +7180,22 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>26.89</v>
+        <v>242.05</v>
       </c>
       <c r="D282" t="n">
-        <v>36.55</v>
+        <v>271.7</v>
       </c>
       <c r="E282" t="n">
-        <v>35.92</v>
+        <v>12.25</v>
       </c>
       <c r="F282" t="n">
-        <v>-0.01787</v>
+        <v>0.65637</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>IEX</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7204,22 +7204,22 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>191.83</v>
+        <v>26.89</v>
       </c>
       <c r="D283" t="n">
-        <v>230.08</v>
+        <v>36.55</v>
       </c>
       <c r="E283" t="n">
-        <v>19.94</v>
+        <v>35.92</v>
       </c>
       <c r="F283" t="n">
-        <v>1.05802</v>
+        <v>-0.01787</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>MGA</t>
+          <t>IEX</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7228,22 +7228,22 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>54.13</v>
+        <v>191.83</v>
       </c>
       <c r="D284" t="n">
-        <v>65</v>
+        <v>230.08</v>
       </c>
       <c r="E284" t="n">
-        <v>20.08</v>
+        <v>19.94</v>
       </c>
       <c r="F284" t="n">
-        <v>-0.60185</v>
+        <v>1.05802</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>MGA</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7252,22 +7252,22 @@
         </is>
       </c>
       <c r="C285" t="n">
-        <v>468.72</v>
+        <v>54.13</v>
       </c>
       <c r="D285" t="n">
-        <v>916.83</v>
+        <v>65</v>
       </c>
       <c r="E285" t="n">
-        <v>95.59999999999999</v>
+        <v>20.08</v>
       </c>
       <c r="F285" t="n">
-        <v>26.11488</v>
+        <v>-0.60185</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>VTRS</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7276,22 +7276,22 @@
         </is>
       </c>
       <c r="C286" t="n">
-        <v>13.16</v>
+        <v>265.47</v>
       </c>
       <c r="D286" t="n">
-        <v>17.83</v>
+        <v>325.77</v>
       </c>
       <c r="E286" t="n">
-        <v>35.49</v>
+        <v>22.71</v>
       </c>
       <c r="F286" t="n">
-        <v>0.21412</v>
+        <v>2.91075</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>CRBG</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7300,22 +7300,22 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>24.11</v>
+        <v>468.72</v>
       </c>
       <c r="D287" t="n">
-        <v>34.87</v>
+        <v>916.83</v>
       </c>
       <c r="E287" t="n">
-        <v>44.63</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="F287" t="n">
-        <v>0.06254999999999999</v>
+        <v>26.11488</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>VTRS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7324,22 +7324,22 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>109.38</v>
+        <v>13.16</v>
       </c>
       <c r="D288" t="n">
-        <v>261.93</v>
+        <v>17.83</v>
       </c>
       <c r="E288" t="n">
-        <v>139.47</v>
+        <v>35.49</v>
       </c>
       <c r="F288" t="n">
-        <v>10.11375</v>
+        <v>0.21412</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>CRBG</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7348,22 +7348,22 @@
         </is>
       </c>
       <c r="C289" t="n">
-        <v>133.15</v>
+        <v>24.11</v>
       </c>
       <c r="D289" t="n">
-        <v>150.2</v>
+        <v>34.87</v>
       </c>
       <c r="E289" t="n">
-        <v>12.81</v>
+        <v>44.63</v>
       </c>
       <c r="F289" t="n">
-        <v>1.3686</v>
+        <v>0.06254999999999999</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7372,22 +7372,22 @@
         </is>
       </c>
       <c r="C290" t="n">
-        <v>555.5700000000001</v>
+        <v>109.38</v>
       </c>
       <c r="D290" t="n">
-        <v>649.13</v>
+        <v>261.94</v>
       </c>
       <c r="E290" t="n">
-        <v>16.84</v>
+        <v>139.48</v>
       </c>
       <c r="F290" t="n">
-        <v>3.9969</v>
+        <v>10.11423</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>HLT</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7396,22 +7396,22 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>302.16</v>
+        <v>133.15</v>
       </c>
       <c r="D291" t="n">
-        <v>313.96</v>
+        <v>150.2</v>
       </c>
       <c r="E291" t="n">
-        <v>3.91</v>
+        <v>12.81</v>
       </c>
       <c r="F291" t="n">
-        <v>-0.28977</v>
+        <v>1.3686</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7420,22 +7420,22 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>710.8</v>
+        <v>555.5700000000001</v>
       </c>
       <c r="D292" t="n">
-        <v>1777.8</v>
+        <v>649.13</v>
       </c>
       <c r="E292" t="n">
-        <v>150.11</v>
+        <v>16.84</v>
       </c>
       <c r="F292" t="n">
-        <v>62.27622</v>
+        <v>3.9969</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>MFC</t>
+          <t>HLT</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7444,22 +7444,22 @@
         </is>
       </c>
       <c r="C293" t="n">
-        <v>35.22</v>
+        <v>302.16</v>
       </c>
       <c r="D293" t="n">
-        <v>43.86</v>
+        <v>313.96</v>
       </c>
       <c r="E293" t="n">
-        <v>24.53</v>
+        <v>3.91</v>
       </c>
       <c r="F293" t="n">
-        <v>0.02451</v>
+        <v>-0.28977</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7468,22 +7468,22 @@
         </is>
       </c>
       <c r="C294" t="n">
-        <v>118.92</v>
+        <v>710.8</v>
       </c>
       <c r="D294" t="n">
-        <v>164.41</v>
+        <v>1777.8</v>
       </c>
       <c r="E294" t="n">
-        <v>38.25</v>
+        <v>150.11</v>
       </c>
       <c r="F294" t="n">
-        <v>2.81053</v>
+        <v>62.27622</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MFC</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7492,40 +7492,40 @@
         </is>
       </c>
       <c r="C295" t="n">
-        <v>178.1</v>
+        <v>35.22</v>
       </c>
       <c r="D295" t="n">
-        <v>225.07</v>
+        <v>43.86</v>
       </c>
       <c r="E295" t="n">
-        <v>26.37</v>
+        <v>24.53</v>
       </c>
       <c r="F295" t="n">
-        <v>2.14735</v>
+        <v>0.02451</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>MOG-B</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C296" t="n">
-        <v>298.49</v>
+        <v>178.1</v>
       </c>
       <c r="D296" t="n">
-        <v>392.72</v>
+        <v>225.07</v>
       </c>
       <c r="E296" t="n">
-        <v>31.57</v>
+        <v>26.37</v>
       </c>
       <c r="F296" t="n">
-        <v>2.31567</v>
+        <v>2.14735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>